<commit_message>
Polish class roster responsiveness
</commit_message>
<xml_diff>
--- a/outputs/live-progress-tracker/SharpStudy-Live-Progress-Tracker.xlsx
+++ b/outputs/live-progress-tracker/SharpStudy-Live-Progress-Tracker.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3bb204cd3f4a4cb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directive Register" sheetId="2" r:id="R91c9b56952da4042"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Register" sheetId="3" r:id="R70e253d984fb4792"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Register" sheetId="4" r:id="Rc3c0e2f85e874a6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Issues" sheetId="5" r:id="R023db328e2d04f8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Evidence" sheetId="6" r:id="R22e7258cbcb54217"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="7" r:id="R628fd486e3f745dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Protocol" sheetId="8" r:id="R9ebb1803549a4354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R274026d04af243ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directive Register" sheetId="2" r:id="R74be0f75ff5142c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Register" sheetId="3" r:id="Rf027f983996949dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Register" sheetId="4" r:id="R87009986c34d43c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Issues" sheetId="5" r:id="Re54f1f01eee04ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Evidence" sheetId="6" r:id="R933069ad131241e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="7" r:id="R51b389f2611d4436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Protocol" sheetId="8" r:id="Re5ca74fc9e9a42d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -175,7 +175,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="124">
+  <x:cellXfs count="123">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -392,6 +392,30 @@
     <x:xf numFmtId="0" fontId="3" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -400,33 +424,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -775,7 +772,7 @@
       </x:c>
       <x:c r="E6" s="22" t="n">
         <x:f>COUNTIF('Feature Register'!$D$2:$D$80,D6)+COUNTIF('Directive Register'!$D$2:$D$80,D6)+COUNTIF('Sprint Register'!$E$2:$E$80,D6)+COUNTIF('Open Issues'!$D$2:$D$80,D6)</x:f>
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G6" s="34" t="str">
         <x:v>P1</x:v>
@@ -819,7 +816,7 @@
       </x:c>
       <x:c r="E8" s="22" t="n">
         <x:f>COUNTIF('Feature Register'!$D$2:$D$80,D8)+COUNTIF('Directive Register'!$D$2:$D$80,D8)+COUNTIF('Sprint Register'!$E$2:$E$80,D8)+COUNTIF('Open Issues'!$D$2:$D$80,D8)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>P3</x:v>
@@ -841,7 +838,7 @@
       </x:c>
       <x:c r="E9" s="22" t="n">
         <x:f>COUNTIF('Feature Register'!$D$2:$D$80,D9)+COUNTIF('Directive Register'!$D$2:$D$80,D9)+COUNTIF('Sprint Register'!$E$2:$E$80,D9)+COUNTIF('Open Issues'!$D$2:$D$80,D9)</x:f>
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1664,13 +1661,13 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="F14" s="55" t="str">
-        <x:v>Collapsed long tables, compact actions, dashboard chart work, modal fixes.</x:v>
+        <x:v>Collapsed long tables, compact actions, dashboard chart work, modal fixes, and responsive class roster cards.</x:v>
       </x:c>
       <x:c r="G14" s="55" t="str">
         <x:v>More visual/device review needed.</x:v>
       </x:c>
       <x:c r="H14" s="60" t="str">
-        <x:v>src/styles.css</x:v>
+        <x:v>src/App.jsx; src/styles.css</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2191,7 +2188,7 @@
         <x:v>src/App.jsx; SCHOOL_PILOT_REVIEW.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A14" s="59" t="str">
         <x:v>F010</x:v>
       </x:c>
@@ -2201,23 +2198,23 @@
       <x:c r="C14" s="55" t="str">
         <x:v>Teacher</x:v>
       </x:c>
-      <x:c r="D14" s="82" t="str">
-        <x:v>Needs Polish</x:v>
+      <x:c r="D14" s="67" t="str">
+        <x:v>Mostly Complete</x:v>
       </x:c>
       <x:c r="E14" s="82" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F14" s="55" t="str">
-        <x:v>Class page lists students with rank, mastery, assignment state, last active, and support signals.</x:v>
+        <x:v>Class page lists students with rank, readiness, assignment state, last active, and support signals. Main roster now wraps on desktop and becomes labelled row cards below tablet width.</x:v>
       </x:c>
       <x:c r="G14" s="55" t="str">
-        <x:v>Avoid crowded tables and reduce columns on smaller screens.</x:v>
+        <x:v>Needs live visual/device review with real class data.</x:v>
       </x:c>
       <x:c r="H14" s="60" t="str">
         <x:v>src/App.jsx; src/styles.css; LIVE_HANDOVER.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="15" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A15" s="59" t="str">
         <x:v>F011</x:v>
       </x:c>
@@ -2234,10 +2231,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F15" s="55" t="str">
-        <x:v>Teacher can open a student view with topic breakdown, support state, and parents' evening review.</x:v>
+        <x:v>Teacher can open a student view with topic breakdown, support state, and parents' evening review. Modal now locks body/html scroll and snaps opened content to the top.</x:v>
       </x:c>
       <x:c r="G15" s="55" t="str">
-        <x:v>Needs visual smoke for modal position/overlay issues.</x:v>
+        <x:v>Needs live visual smoke for edge-case overlay issues.</x:v>
       </x:c>
       <x:c r="H15" s="60" t="str">
         <x:v>src/App.jsx</x:v>
@@ -3151,7 +3148,7 @@
         <x:v>User notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="59" t="str">
         <x:v>I006</x:v>
       </x:c>
@@ -3161,23 +3158,23 @@
       <x:c r="C10" s="55" t="str">
         <x:v>UX</x:v>
       </x:c>
-      <x:c r="D10" s="82" t="str">
-        <x:v>Needs Polish</x:v>
+      <x:c r="D10" s="67" t="str">
+        <x:v>Mostly Complete</x:v>
       </x:c>
       <x:c r="E10" s="82" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F10" s="55" t="str">
-        <x:v>Long tables can become cramped or hide important columns.</x:v>
+        <x:v>Main class roster now avoids horizontal scroll, wraps desktop content, and becomes labelled row cards below tablet width.</x:v>
       </x:c>
       <x:c r="G10" s="55" t="str">
-        <x:v>Continue responsive table audits.</x:v>
+        <x:v>Manual device/browser review still required.</x:v>
       </x:c>
       <x:c r="H10" s="60" t="str">
-        <x:v>src/styles.css</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+        <x:v>src/App.jsx; src/styles.css</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="59" t="str">
         <x:v>I007</x:v>
       </x:c>
@@ -3187,20 +3184,20 @@
       <x:c r="C11" s="55" t="str">
         <x:v>UX</x:v>
       </x:c>
-      <x:c r="D11" s="103" t="str">
-        <x:v>Needs Manual Review</x:v>
+      <x:c r="D11" s="67" t="str">
+        <x:v>Mostly Complete</x:v>
       </x:c>
       <x:c r="E11" s="82" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F11" s="55" t="str">
-        <x:v>Past notes mention modal opening low/overlaying buttons.</x:v>
+        <x:v>Modal opening now scrolls the selected dialog to the top and locks both body and html scroll while open.</x:v>
       </x:c>
       <x:c r="G11" s="55" t="str">
-        <x:v>Visual smoke required.</x:v>
+        <x:v>Manual visual smoke still required.</x:v>
       </x:c>
       <x:c r="H11" s="60" t="str">
-        <x:v>LIVE_HANDOVER.md</x:v>
+        <x:v>src/App.jsx; LIVE_HANDOVER.md</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3265,7 +3262,7 @@
       <x:c r="C14" s="55" t="str">
         <x:v>Security/Backend</x:v>
       </x:c>
-      <x:c r="D14" s="107" t="str">
+      <x:c r="D14" s="103" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="E14" s="91" t="str">
@@ -3291,7 +3288,7 @@
       <x:c r="C15" s="55" t="str">
         <x:v>Security/Backend</x:v>
       </x:c>
-      <x:c r="D15" s="107" t="str">
+      <x:c r="D15" s="103" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="E15" s="91" t="str">
@@ -3317,7 +3314,7 @@
       <x:c r="C16" s="55" t="str">
         <x:v>Operations</x:v>
       </x:c>
-      <x:c r="D16" s="107" t="str">
+      <x:c r="D16" s="103" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="E16" s="82" t="str">
@@ -3447,7 +3444,7 @@
       <x:c r="C21" s="55" t="str">
         <x:v>Learning/AI</x:v>
       </x:c>
-      <x:c r="D21" s="107" t="str">
+      <x:c r="D21" s="103" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="E21" s="87" t="str">
@@ -3473,7 +3470,7 @@
       <x:c r="C22" s="55" t="str">
         <x:v>Business</x:v>
       </x:c>
-      <x:c r="D22" s="107" t="str">
+      <x:c r="D22" s="103" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="E22" s="82" t="str">
@@ -3502,7 +3499,7 @@
       <x:c r="D23" s="95" t="str">
         <x:v>Planned</x:v>
       </x:c>
-      <x:c r="E23" s="111" t="str">
+      <x:c r="E23" s="107" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="F23" s="62" t="str">
@@ -3712,7 +3709,7 @@
       <x:c r="C9" s="55" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="D9" s="102" t="str">
+      <x:c r="D9" s="110" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="E9" s="55" t="str">
@@ -3735,7 +3732,7 @@
       <x:c r="C10" s="55" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="D10" s="102" t="str">
+      <x:c r="D10" s="110" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="E10" s="55" t="str">
@@ -3781,7 +3778,7 @@
       <x:c r="C12" s="62" t="str">
         <x:v>Manual</x:v>
       </x:c>
-      <x:c r="D12" s="114" t="str">
+      <x:c r="D12" s="113" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="E12" s="62" t="str">
@@ -4047,155 +4044,155 @@
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="116" t="str">
+      <x:c r="A4" s="115" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="B4" s="117" t="str">
+      <x:c r="B4" s="116" t="str">
         <x:v>Action</x:v>
       </x:c>
-      <x:c r="C4" s="117" t="str">
+      <x:c r="C4" s="116" t="str">
         <x:v>Applies To</x:v>
       </x:c>
-      <x:c r="D4" s="117" t="str">
+      <x:c r="D4" s="116" t="str">
         <x:v>Required Evidence</x:v>
       </x:c>
-      <x:c r="E4" s="118" t="str">
+      <x:c r="E4" s="117" t="str">
         <x:v>Commit Rule</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="119" t="str">
+      <x:c r="A5" s="118" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B5" s="115" t="str">
+      <x:c r="B5" s="114" t="str">
         <x:v>Update the relevant row status and remaining work.</x:v>
       </x:c>
-      <x:c r="C5" s="115" t="str">
+      <x:c r="C5" s="114" t="str">
         <x:v>All registers</x:v>
       </x:c>
-      <x:c r="D5" s="115" t="str">
+      <x:c r="D5" s="114" t="str">
         <x:v>Reference file, commit, test output, or manual test note.</x:v>
       </x:c>
-      <x:c r="E5" s="120" t="str">
+      <x:c r="E5" s="119" t="str">
         <x:v>Do not leave status stale.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A6" s="119" t="str">
+      <x:c r="A6" s="118" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B6" s="115" t="str">
+      <x:c r="B6" s="114" t="str">
         <x:v>Add new feature/subfeature rows rather than hiding work inside broad items.</x:v>
       </x:c>
-      <x:c r="C6" s="115" t="str">
+      <x:c r="C6" s="114" t="str">
         <x:v>Feature Register</x:v>
       </x:c>
-      <x:c r="D6" s="115" t="str">
+      <x:c r="D6" s="114" t="str">
         <x:v>Short evidence path.</x:v>
       </x:c>
-      <x:c r="E6" s="120" t="str">
+      <x:c r="E6" s="119" t="str">
         <x:v>One row per meaningful subfeature.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A7" s="119" t="str">
+      <x:c r="A7" s="118" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B7" s="115" t="str">
+      <x:c r="B7" s="114" t="str">
         <x:v>Update Dashboard summary formulas only if row ranges are expanded beyond row 80.</x:v>
       </x:c>
-      <x:c r="C7" s="115" t="str">
+      <x:c r="C7" s="114" t="str">
         <x:v>Dashboard</x:v>
       </x:c>
-      <x:c r="D7" s="115" t="str">
+      <x:c r="D7" s="114" t="str">
         <x:v>Formula scan passes.</x:v>
       </x:c>
-      <x:c r="E7" s="120" t="str">
+      <x:c r="E7" s="119" t="str">
         <x:v>Keep formulas auditable.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="119" t="str">
+      <x:c r="A8" s="118" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B8" s="115" t="str">
+      <x:c r="B8" s="114" t="str">
         <x:v>Update LIVE_HANDOVER.md with the same status change.</x:v>
       </x:c>
-      <x:c r="C8" s="115" t="str">
+      <x:c r="C8" s="114" t="str">
         <x:v>Handover</x:v>
       </x:c>
-      <x:c r="D8" s="115" t="str">
+      <x:c r="D8" s="114" t="str">
         <x:v>Handover change log.</x:v>
       </x:c>
-      <x:c r="E8" s="120" t="str">
+      <x:c r="E8" s="119" t="str">
         <x:v>Tracker and handover must agree.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A9" s="119" t="str">
+      <x:c r="A9" s="118" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B9" s="115" t="str">
+      <x:c r="B9" s="114" t="str">
         <x:v>Run npm test, npm run build, and npm run test:rules when code/rules changed.</x:v>
       </x:c>
-      <x:c r="C9" s="115" t="str">
+      <x:c r="C9" s="114" t="str">
         <x:v>Code sprints</x:v>
       </x:c>
-      <x:c r="D9" s="115" t="str">
+      <x:c r="D9" s="114" t="str">
         <x:v>Test Evidence row updated.</x:v>
       </x:c>
-      <x:c r="E9" s="120" t="str">
+      <x:c r="E9" s="119" t="str">
         <x:v>Docs-only changes may use lighter checks.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A10" s="119" t="str">
+      <x:c r="A10" s="118" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B10" s="115" t="str">
+      <x:c r="B10" s="114" t="str">
         <x:v>Run manual production smoke checks for live Firebase/browser-only items.</x:v>
       </x:c>
-      <x:c r="C10" s="115" t="str">
+      <x:c r="C10" s="114" t="str">
         <x:v>Manual QA</x:v>
       </x:c>
-      <x:c r="D10" s="115" t="str">
+      <x:c r="D10" s="114" t="str">
         <x:v>PRODUCTION_SMOKE_TEST_2026-07-29.md.</x:v>
       </x:c>
-      <x:c r="E10" s="120" t="str">
+      <x:c r="E10" s="119" t="str">
         <x:v>Do not mark manual items complete from code inspection.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="119" t="str">
+      <x:c r="A11" s="118" t="str">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B11" s="115" t="str">
+      <x:c r="B11" s="114" t="str">
         <x:v>Commit and push tracker updates with the related sprint.</x:v>
       </x:c>
-      <x:c r="C11" s="115" t="str">
+      <x:c r="C11" s="114" t="str">
         <x:v>All</x:v>
       </x:c>
-      <x:c r="D11" s="115" t="str">
+      <x:c r="D11" s="114" t="str">
         <x:v>Git commit hash.</x:v>
       </x:c>
-      <x:c r="E11" s="120" t="str">
+      <x:c r="E11" s="119" t="str">
         <x:v>Keep GitHub as source of truth.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A12" s="121" t="str">
+      <x:c r="A12" s="120" t="str">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B12" s="122" t="str">
+      <x:c r="B12" s="121" t="str">
         <x:v>Create a physical backup after major sprint groups if Jonah asks for a save.</x:v>
       </x:c>
-      <x:c r="C12" s="122" t="str">
+      <x:c r="C12" s="121" t="str">
         <x:v>Operations</x:v>
       </x:c>
-      <x:c r="D12" s="122" t="str">
+      <x:c r="D12" s="121" t="str">
         <x:v>app-saves bundle/zip path.</x:v>
       </x:c>
-      <x:c r="E12" s="123" t="str">
+      <x:c r="E12" s="122" t="str">
         <x:v>Do not include secrets.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Polish student dashboard clarity
</commit_message>
<xml_diff>
--- a/outputs/live-progress-tracker/SharpStudy-Live-Progress-Tracker.xlsx
+++ b/outputs/live-progress-tracker/SharpStudy-Live-Progress-Tracker.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd4984b7f035c4a1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directive Register" sheetId="2" r:id="Reb849c4acbb34d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Register" sheetId="3" r:id="Rf84a4fda18fe4ab3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Register" sheetId="4" r:id="R64da33b124ea4f31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Issues" sheetId="5" r:id="Rd2898200c488490e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Evidence" sheetId="6" r:id="R807bfb215db44e33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="7" r:id="R9ba197c7d3814758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Protocol" sheetId="8" r:id="R7887c23096264688"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R88730318360c4d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directive Register" sheetId="2" r:id="R024e3c94b4b04473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Register" sheetId="3" r:id="Rae5cf856101a4eed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Register" sheetId="4" r:id="R2b641948101548e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Issues" sheetId="5" r:id="R2d62750825c84d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Evidence" sheetId="6" r:id="R3ab56249278a4a21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="7" r:id="R536ef44838b144bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Protocol" sheetId="8" r:id="R6f629ba512ef47c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -624,14 +624,14 @@
         <x:v>Latest sprint</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Report filter clarity pass; see Git history for exact commit hash</x:v>
+        <x:v>Student dashboard clarity pass; see Git history for exact commit hash</x:v>
       </x:c>
       <x:c r="D6" s="19" t="str">
         <x:v>Mostly Complete</x:v>
       </x:c>
       <x:c r="E6" s="15" t="n">
         <x:f>COUNTIF('Feature Register'!$D$2:$D$80,D6)+COUNTIF('Directive Register'!$D$2:$D$80,D6)+COUNTIF('Sprint Register'!$E$2:$E$80,D6)+COUNTIF('Open Issues'!$D$2:$D$80,D6)</x:f>
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
         <x:v>P1</x:v>
@@ -641,12 +641,12 @@
         <x:v>25</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="11" t="str">
         <x:v>Latest checks</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>npm test, npm run build, npm run test:rules all passed on 2026-07-30</x:v>
+        <x:v>npm test, npm run build, npm run test:rules all passed on 2026-07-30; browser/device visual review remains manual</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
         <x:v>In Progress</x:v>
@@ -697,7 +697,7 @@
       </x:c>
       <x:c r="E9" s="15" t="n">
         <x:f>COUNTIF('Feature Register'!$D$2:$D$80,D9)+COUNTIF('Directive Register'!$D$2:$D$80,D9)+COUNTIF('Sprint Register'!$E$2:$E$80,D9)+COUNTIF('Open Issues'!$D$2:$D$80,D9)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1520,7 +1520,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="F14" s="47" t="str">
-        <x:v>Collapsed long tables, compact actions, dashboard chart work, modal fixes, responsive class roster cards, and clearer report filter guidance.</x:v>
+        <x:v>Collapsed long tables, compact actions, dashboard chart work, modal fixes, responsive class roster cards, clearer report filter guidance, and reduced-clutter student dashboard ordering.</x:v>
       </x:c>
       <x:c r="G14" s="47" t="str">
         <x:v>More visual/device review needed.</x:v>
@@ -1813,7 +1813,7 @@
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A5" s="47" t="str">
         <x:v>F001</x:v>
       </x:c>
@@ -1830,13 +1830,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F5" s="47" t="str">
-        <x:v>Student dashboard includes memory decay, active assignments, quiz, Blitz, Match, Learn, Info, leaderboard, teacher messages, and class joining.</x:v>
+        <x:v>Student dashboard now opens as the main menu with memory decay, coverage, mastery, active assignment count, one recommended next step, assignments, quiz, Blitz, Match, Learn, Info, leaderboard, teacher messages, class joining, and collapsible subsection progress.</x:v>
       </x:c>
       <x:c r="G5" s="47" t="str">
-        <x:v>Needs clutter reduction and subsection progress-bar polish from latest UX notes.</x:v>
+        <x:v>Needs manual student/device review to confirm the reduced-clutter layout works in the deployed app.</x:v>
       </x:c>
       <x:c r="H5" s="47" t="str">
-        <x:v>src/App.jsx; LIVE_HANDOVER.md</x:v>
+        <x:v>src/App.jsx; src/styles.css; LIVE_HANDOVER.md</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2981,7 +2981,7 @@
         <x:v>src/App.jsx; LIVE_HANDOVER.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="9" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A9" s="47" t="str">
         <x:v>I005</x:v>
       </x:c>
@@ -2991,20 +2991,20 @@
       <x:c r="C9" s="47" t="str">
         <x:v>UX</x:v>
       </x:c>
-      <x:c r="D9" s="63" t="str">
-        <x:v>Needs Polish</x:v>
+      <x:c r="D9" s="51" t="str">
+        <x:v>Mostly Complete</x:v>
       </x:c>
       <x:c r="E9" s="63" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F9" s="47" t="str">
-        <x:v>Dashboard should become main menu with memory bar/subsection progress and class join below.</x:v>
+        <x:v>Main dashboard now includes a recommended next step, keeps assignments above class joining/messages, collapses teacher messages by default, and keeps subsection progress available without forcing it open in every normal case.</x:v>
       </x:c>
       <x:c r="G9" s="47" t="str">
-        <x:v>Plan UX sprint.</x:v>
+        <x:v>Manual student UX and phone/laptop visual review still required.</x:v>
       </x:c>
       <x:c r="H9" s="47" t="str">
-        <x:v>User notes</x:v>
+        <x:v>src/App.jsx; src/styles.css</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3486,7 +3486,7 @@
         <x:v>2026-07-30</x:v>
       </x:c>
       <x:c r="G5" s="47" t="str">
-        <x:v>Latest after email-verification sprint.</x:v>
+        <x:v>Latest after student dashboard clarity sprint.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -3503,13 +3503,13 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="E6" s="47" t="str">
-        <x:v>Vite build passed; main app chunk 434.04 kB</x:v>
+        <x:v>Vite build passed; main app chunk 435.52 kB</x:v>
       </x:c>
       <x:c r="F6" s="47" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
       <x:c r="G6" s="47" t="str">
-        <x:v>React/Firebase chunks split.</x:v>
+        <x:v>React/Firebase chunks split; latest after dashboard clarity sprint.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -3555,7 +3555,7 @@
         <x:v>2026-07-30</x:v>
       </x:c>
       <x:c r="G8" s="47" t="str">
-        <x:v>Report filter clarity sprint.</x:v>
+        <x:v>Student dashboard clarity sprint.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">

</xml_diff>